<commit_message>
Atualiza conversa estudante 48: icaropda@outlook.com com historico ENADE/Gini
</commit_message>
<xml_diff>
--- a/interacoes_estudantes.xlsx
+++ b/interacoes_estudantes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo.lima\Desktop\PBIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C62F7A-EF25-4977-9189-450CC02DFED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BFEEFA3-0696-49DE-9D84-C1D5CE8E65EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="205">
   <si>
     <t>Estudante</t>
   </si>
@@ -628,6 +628,18 @@
   </si>
   <si>
     <t>Maria Torres - free</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Precisa ser descosiderado da conta</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>2x no email</t>
+  </si>
+  <si>
+    <t>colcoar o icaropda@outlook.com</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -1058,7 +1070,7 @@
     <col min="4" max="4" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1069,7 +1081,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1079,8 +1091,11 @@
       <c r="C2" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1090,8 +1105,11 @@
       <c r="C3" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1101,8 +1119,11 @@
       <c r="C4" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1112,8 +1133,11 @@
       <c r="C5" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1123,8 +1147,11 @@
       <c r="C6" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1134,8 +1161,11 @@
       <c r="C7" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1145,8 +1175,11 @@
       <c r="C8" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1156,8 +1189,11 @@
       <c r="C9" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1165,10 +1201,13 @@
         <v>19</v>
       </c>
       <c r="C10" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1178,8 +1217,11 @@
       <c r="C11" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1187,10 +1229,13 @@
         <v>23</v>
       </c>
       <c r="C12" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1200,8 +1245,11 @@
       <c r="C13" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1211,8 +1259,11 @@
       <c r="C14" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1222,8 +1273,11 @@
       <c r="C15" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1233,8 +1287,11 @@
       <c r="C16" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1244,8 +1301,11 @@
       <c r="C17" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1255,8 +1315,11 @@
       <c r="C18" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1266,8 +1329,11 @@
       <c r="C19" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1277,8 +1343,11 @@
       <c r="C20" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -1288,8 +1357,11 @@
       <c r="C21" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -1299,8 +1371,11 @@
       <c r="C22" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -1310,8 +1385,14 @@
       <c r="C23" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>202</v>
+      </c>
+      <c r="F23" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -1321,8 +1402,11 @@
       <c r="C24" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -1332,8 +1416,11 @@
       <c r="C25" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -1343,8 +1430,11 @@
       <c r="C26" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -1354,8 +1444,11 @@
       <c r="C27" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -1365,8 +1458,11 @@
       <c r="C28" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -1376,8 +1472,11 @@
       <c r="C29" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -1387,8 +1486,11 @@
       <c r="C30" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -1398,8 +1500,11 @@
       <c r="C31" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E31" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -1409,8 +1514,11 @@
       <c r="C32" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>64</v>
       </c>
@@ -1420,8 +1528,14 @@
       <c r="C33" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
+        <v>202</v>
+      </c>
+      <c r="F33" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>66</v>
       </c>
@@ -1431,8 +1545,11 @@
       <c r="C34" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -1442,8 +1559,11 @@
       <c r="C35" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>70</v>
       </c>
@@ -1453,8 +1573,11 @@
       <c r="C36" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>72</v>
       </c>
@@ -1464,8 +1587,11 @@
       <c r="C37" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E37" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -1475,8 +1601,11 @@
       <c r="C38" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>76</v>
       </c>
@@ -1486,8 +1615,14 @@
       <c r="C39" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E39" t="s">
+        <v>202</v>
+      </c>
+      <c r="F39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>78</v>
       </c>
@@ -1497,8 +1632,11 @@
       <c r="C40" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E40" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>80</v>
       </c>
@@ -1509,7 +1647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>82</v>
       </c>
@@ -1517,10 +1655,10 @@
         <v>83</v>
       </c>
       <c r="C42" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -1528,10 +1666,10 @@
         <v>85</v>
       </c>
       <c r="C43" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>86</v>
       </c>
@@ -1539,10 +1677,10 @@
         <v>87</v>
       </c>
       <c r="C44" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>88</v>
       </c>
@@ -1550,10 +1688,10 @@
         <v>89</v>
       </c>
       <c r="C45" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>90</v>
       </c>
@@ -1561,10 +1699,10 @@
         <v>91</v>
       </c>
       <c r="C46" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>92</v>
       </c>
@@ -1572,10 +1710,10 @@
         <v>93</v>
       </c>
       <c r="C47" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -1583,10 +1721,10 @@
         <v>95</v>
       </c>
       <c r="C48" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>96</v>
       </c>
@@ -1597,7 +1735,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>98</v>
       </c>
@@ -1607,8 +1745,14 @@
       <c r="C50" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F50" t="s">
+        <v>201</v>
+      </c>
+      <c r="J50" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>100</v>
       </c>
@@ -1618,8 +1762,11 @@
       <c r="C51" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E51" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -1629,8 +1776,11 @@
       <c r="C52" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E52" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -1640,8 +1790,11 @@
       <c r="C53" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>106</v>
       </c>
@@ -1651,8 +1804,11 @@
       <c r="C54" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E54" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>108</v>
       </c>
@@ -1663,7 +1819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>110</v>
       </c>
@@ -1674,7 +1830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>112</v>
       </c>
@@ -1685,7 +1841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>114</v>
       </c>
@@ -1696,7 +1852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>116</v>
       </c>
@@ -1707,7 +1863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>118</v>
       </c>
@@ -1718,7 +1874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>120</v>
       </c>
@@ -1729,7 +1885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>122</v>
       </c>
@@ -1737,10 +1893,10 @@
         <v>123</v>
       </c>
       <c r="C62" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>124</v>
       </c>
@@ -1748,10 +1904,10 @@
         <v>125</v>
       </c>
       <c r="C63" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>126</v>
       </c>
@@ -1803,7 +1959,7 @@
         <v>135</v>
       </c>
       <c r="C68" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1825,7 +1981,7 @@
         <v>139</v>
       </c>
       <c r="C70" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -2078,7 +2234,7 @@
         <v>184</v>
       </c>
       <c r="C93" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>